<commit_message>
feat: update PC build budget with new components and pricing, enhance compatibility notes
</commit_message>
<xml_diff>
--- a/pc_build_budget.xlsx
+++ b/pc_build_budget.xlsx
@@ -2,60 +2,236 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="23040" windowHeight="9000" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="PC Build Budget" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;Rp &quot;#,##0"/>
+    <numFmt numFmtId="165" formatCode="_-&quot;Rp&quot;* #,##0.00_-;\-&quot;Rp&quot;* #,##0.00_-;_-&quot;Rp&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="_-&quot;Rp&quot;* #,##0_-;\-&quot;Rp&quot;* #,##0_-;_-&quot;Rp&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="6">
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
+  <fonts count="28">
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
       <name val="Calibri"/>
+      <charset val="134"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="16"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="16"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <i val="1"/>
-      <color rgb="00595959"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
+      <color rgb="FF595959"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <b val="1"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="Calibri"/>
+      <charset val="134"/>
       <b val="1"/>
-      <color rgb="001F4E78"/>
+      <color rgb="FF1F4E78"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF800080"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="18"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <i val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="15"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="13"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF3F3F76"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FF3F3F3F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF006100"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF9C0006"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF9C6500"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color theme="0"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="37">
     <fill>
       <patternFill/>
     </fill>
@@ -64,30 +240,216 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-        <bgColor rgb="001F4E78"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="002F5597"/>
-        <bgColor rgb="002F5597"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
-        <bgColor rgb="00F2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
-        <bgColor rgb="00D9E1F2"/>
+        <fgColor rgb="FF1F4E78"/>
+        <bgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2F5597"/>
+        <bgColor rgb="FF2F5597"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9E1F2"/>
+        <bgColor rgb="FFD9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -97,57 +459,298 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </left>
       <right style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </right>
       <top style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </bottom>
-    </border>
-    <border>
-      <top style="thin">
-        <color rgb="001F4E78"/>
-      </top>
-      <bottom style="double">
-        <color rgb="001F4E78"/>
-      </bottom>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="001F4E78"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right/>
       <top style="thin">
-        <color rgb="001F4E78"/>
+        <color rgb="FF1F4E78"/>
       </top>
       <bottom style="double">
-        <color rgb="001F4E78"/>
+        <color rgb="FF1F4E78"/>
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF1F4E78"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="49">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="9" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="9" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="34" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="35" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="36" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -157,6 +760,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="6"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -164,17 +768,74 @@
     <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="49">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -527,7 +1188,6 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -537,14 +1197,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="45" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="76.2222222222222" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
@@ -553,314 +1214,379 @@
           <t>🖥️ PC Build &amp; Budget Tracker - learn-with-runa</t>
         </is>
       </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Owner: User | Assistant: Runa Shirakawa | Status: In Progress ⏳</t>
         </is>
       </c>
     </row>
     <row r="4" ht="25" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Component Name</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Price (IDR)</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Notes / Compatibility</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>LINK</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="4" t="n">
+      <c r="A5" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>CPU</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>AMD Ryzen 5 5500</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="n">
-        <v>1600000</v>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>6 Cores 12 Threads, Socket AM4, PCIe 3.0</t>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>AMD Ryzen 5 5600</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="n">
+        <v>2139000</v>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>6 Cores 12 Threads, Socket AM4, PCIe 4.0</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>https://shopee.co.id/AMD-CPU-PROCESSOR-RYZEN-5-5600-(6C-12T-3.5-4.4GHZ)-32MB-CACHE-TDP-65W-AM4-TRAY-i.1111772338.49509062565?extraParams=%7B%22display_model_id%22%3A430801512564%2C%22model_selection_logic%22%3A3%7D</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="7" t="n">
+      <c r="A6" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>GPU</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
         <is>
           <t>NVIDIA GTX 1050 Ti</t>
         </is>
       </c>
-      <c r="D6" s="9" t="n">
+      <c r="D6" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>Pake yang sudah ada dulu (Temporary)</t>
         </is>
       </c>
+      <c r="F6" s="11" t="n"/>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="4" t="n">
+      <c r="A7" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Motherboard</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Asrock B450M Steel Legend AM4 RGB</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>1562000</v>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Socket AM4, Micro-ATX, RGB &amp; VRM mantap</t>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Asrock B550M PRO SE AMD AM4 DDR4 WHITE</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="n">
+        <v>1667000</v>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Socket AM4, Micro-ATX</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>https://shopee.co.id/Motherboard-Asrock-B550M-PRO-SE-AMD-AM4-DDR4-i.31995121.42107176365?extraParams=%7B%22display_model_id%22%3A285607805468%2C%22model_selection_logic%22%3A3%7D</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="7" t="n">
+      <c r="A8" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>RAM</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="11" t="inlineStr">
         <is>
           <t>KINGBANK SOARBLADE RGB WHITE 2x16GB (32GB) 3600MHz CL18</t>
         </is>
       </c>
-      <c r="D8" s="9" t="n">
-        <v>3600000</v>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="D8" s="18" t="n">
+        <v>3860000</v>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>Dual Channel 32GB Kit, DDR4 3600MHz, White RGB</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>https://shopee.co.id/RAM-PC-KINGBANK-SOARBLADE-RGB-WHITE-2x16GB-16GBx2-DDR4-(16GB-Kit-of-2-Total-32GB)-3600MHz-CL18-Limited-Lifetime-K5.01.FL04AD9301-i.37363092.44031921635?xptdk=b7b6cd77-1529-43a2-9b10-58987c11af6f</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="4" t="n">
+      <c r="A9" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>Storage (SSD/HDD)</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>TEAM SSD NVME GEN3 MP33 512GB M.2 2280</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>1500000</v>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>NVMe PCIe 3.0 x4, Speed up to 1800 MB/s, Garansi 5 Thn</t>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>SSD NVME 512GB PCIe Gen4x4 SENTINEL 100%/100% (POT 0 Day) Like New</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="n">
+        <v>1100000</v>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>NVMe PCIe Gen4x4 512GB, Health 100%/100% Sentinel (POT 0 Day), Like New</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>https://shopee.co.id/SSD-NVME-512GB-PCIe-Gen4x4-SENTINEL-100-100-(POT-0-Day)-Like-New-i.58275179.50407756227?extraParams=%7B%22display_model_id%22%3A431377608725%2C%22model_selection_logic%22%3A3%7D</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="7" t="n">
+      <c r="A10" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Power Supply (PSU)</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="11" t="inlineStr">
         <is>
           <t>Cooler Master MWE 650 V3 - 650W 80+ BRONZE</t>
         </is>
       </c>
-      <c r="D10" s="9" t="n">
-        <v>700000</v>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="D10" s="18" t="n">
+        <v>795000</v>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>80+ Bronze efficiency, mantap buat build mid-range</t>
+        </is>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>https://shopee.co.id/Cooler-Master-MWE-650-V3-650W-80-BRONZE-i.1120452270.28718225957?xptdk=8611ab72-23d0-4733-9a62-003566b3d231</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="4" t="n">
+      <c r="A11" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Case</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>Tecware VX Trinity M2 M-ATX TG Case White (3x ARGB Fans)</t>
         </is>
       </c>
-      <c r="D11" s="6" t="n">
-        <v>470000</v>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="D11" s="17" t="n">
+        <v>535000</v>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>M-ATX, Tempered Glass, Inc. 3x ARGB Fans White, cocok sama tema White &amp; ARGB</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>https://shopee.co.id/Tecware-VX-Trinity-M2-M-ATX-TG-Case-with-3-x-ARGB-Fans-WHITE-i.24539943.55266903066?xptdk=ed1b3bd4-1851-4ccf-8d87-83db930bca1d</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="7" t="n">
+      <c r="A12" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Cooler</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C12" s="11" t="inlineStr">
         <is>
           <t>COOLMOON AOSOR CPU COOLER T6 DIGITAL 12CM ARGB 6 PIPE White</t>
         </is>
       </c>
-      <c r="D12" s="9" t="n">
-        <v>300000</v>
-      </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="D12" s="18" t="n">
+        <v>323000</v>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
         <is>
           <t>White Air Cooler, 6 Heatpipes, ARGB &amp; Digital Display</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>https://shopee.co.id/COOLMOON-AOSOR-CPU-COOLER-T6-DIGITAL-12CM-ARGB-6-PIPE-i.18361779.48805703004?xptdk=9689ff4b-aabd-45b8-af83-f2587f958324</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="4" t="n">
+      <c r="A13" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Monitor</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>ASRock CL27FFB 27 Inch IPS FHD 144Hz 99% sRGB</t>
         </is>
       </c>
-      <c r="D13" s="6" t="n">
-        <v>1600000</v>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="D13" s="17" t="n">
+        <v>1700000</v>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>27" IPS, FHD (1080p), 144Hz, 99% sRGB</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>https://shopee.co.id/ASRock-CL27FFB-27-Inch-IPS-FHD-144Hz-99-sRGB-Monitor-LED-i.467406516.51017044691?xptdk=d662d7d2-e317-4b3e-b580-87a1273d3f6d</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="7" t="n">
+      <c r="A14" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>Network / Wi-Fi</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>TP-LINK TL-WN881ND Wireless N PCI Express</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="n">
-        <v>150000</v>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>PCIe Wi-Fi Card 300Mbps, 2x Antena 2dBi</t>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>PCIE Wifi Dual Band Bluetooth Qualcomm Atheros Wireless Network Card</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="n">
+        <v>199000</v>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>PCIe Wi-Fi Dual Band 2.4G/5G + Bluetooth (Qualcomm Atheros)</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>https://shopee.co.id/PCIE-Wifi-Dual-Band-Bluetooth-Qualcomm-Atheros-Wireless-Network-Card-i.52470016.15754410597?extraParams=%7B%22display_model_id%22%3A142567595543%2C%22model_selection_logic%22%3A3%7D</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="4" t="n">
+      <c r="A15" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>Accessories / Extra</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>MM-Cyclone Fan ARGB 12cm (3 pcs)</t>
         </is>
       </c>
-      <c r="D15" s="6" t="n">
-        <v>118000</v>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="D15" s="17" t="n">
+        <v>125000</v>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
         <is>
           <t>Fan tambahan ARGB 3pcs</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>https://shopee.co.id/-MM-Cyclone-Kipas-Pendingin-12cm-Kipas-Performa-Tinggi-Kipas-Senyap-Fantasi-ARGB-12-24-Volt-Fan-gen4-Garansi-1-Tahun-i.1744608100.44659068599?xptdk=4514b8c6-3762-4e9e-8877-9d007e979978</t>
         </is>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>Total Estimated Price</t>
         </is>
       </c>
-      <c r="B17" s="13" t="n"/>
-      <c r="C17" s="13" t="n"/>
-      <c r="D17" s="12">
+      <c r="B17" s="14" t="n"/>
+      <c r="C17" s="14" t="n"/>
+      <c r="D17" s="19">
         <f>SUM(D5:D15)</f>
         <v/>
       </c>
-      <c r="E17" s="11" t="n"/>
+      <c r="E17" s="16" t="n"/>
+      <c r="F17" s="16" t="n"/>
     </row>
+    <row r="18" ht="15.15" customHeight="1"/>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
     <mergeCell ref="A17:C17"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" display="https://shopee.co.id/AMD-CPU-PROCESSOR-RYZEN-5-5600-(6C-12T-3.5-4.4GHZ)-32MB-CACHE-TDP-65W-AM4-TRAY-i.1111772338.49509062565?extraParams=%7B%22display_model_id%22%3A430801512564%2C%22model_selection_logic%22%3A3%7D" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>